<commit_message>
Fix invisible column headers in experiment log Excel files
</commit_message>
<xml_diff>
--- a/EXPERIMENT_LOG_AUTOENCODER.xlsx
+++ b/EXPERIMENT_LOG_AUTOENCODER.xlsx
@@ -29,7 +29,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
   <fills count="6">
@@ -41,26 +41,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-        <bgColor rgb="00D9D9D9"/>
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,16 +74,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
     </border>
   </borders>

</xml_diff>